<commit_message>
Update workbook for week of 10/12 with make-ahead sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016abfmfMm3FJdNo4xsxKHTV
</commit_message>
<xml_diff>
--- a/献立表_レシピ_買い物リスト.xlsx
+++ b/献立表_レシピ_買い物リスト.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="献立表" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="レシピ" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="買い物リスト" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="出典・基礎原理" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="作り置き" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="レシピ" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="買い物リスト" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="出典・基礎原理" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -51,6 +52,7 @@
     <font>
       <name val="Meiryo"/>
       <b val="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -92,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -107,8 +109,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -474,38 +475,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>日付</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>曜日</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>朝</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>昼</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>夜</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>間食</t>
         </is>
@@ -514,25 +521,30 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>10/12</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
           <t>月</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>ご飯 / 卵と豆腐の味噌汁 / 納豆</t>
-        </is>
-      </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>鮭おにぎり / ほうれん草のおひたし / みかん</t>
+          <t>ご飯 / 小松菜と油揚げの味噌汁 / 納豆</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>鶏ももと根菜の照り煮 / ご飯 / 味噌汁 / 冷凍ブロッコリー</t>
+          <t>豚の生姜焼き+千切りキャベツ / ご飯 / かぼちゃの煮物</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>鮭のちゃんちゃん焼き / ご飯 / ひじきの煮物</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>ヨーグルト+冷凍ブルーベリー</t>
         </is>
@@ -541,25 +553,30 @@
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
+          <t>10/13</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
           <t>火</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>ご飯 / ゆで卵 / ヨーグルト+ブルーベリー+キウイ</t>
-        </is>
-      </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>基本の親子丼 / ほうれん草のおひたし</t>
+          <t>ご飯 / ゆで卵 / ヨーグルト+冷凍ブルーベリー</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>鯖の塩焼き / 冷奴 / ご飯 / 味噌汁 / 冷凍ブロッコリー</t>
+          <t>けんちん汁 / おにぎり / 小松菜の煮浸し</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>鶏の照り焼き / ブロッコリーとツナのマヨ和え / ご飯</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>バナナ</t>
         </is>
@@ -568,25 +585,30 @@
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>10/14</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
           <t>水</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>トースト / チーズ / バナナ / 牛乳(ブルーベリースムージーも可)</t>
-        </is>
-      </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>豚汁 / おにぎり</t>
+          <t>トースト / チーズ / バナナ / 牛乳</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>照り煮の残り / ほうれん草のおひたし / ご飯</t>
+          <t>照り焼き丼(残り) / 味噌汁</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>豆腐ハンバーグ / 小松菜の煮浸し / ご飯</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>チーズ・ナッツ</t>
         </is>
@@ -595,115 +617,135 @@
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>10/15</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
           <t>木</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>ご飯 / 納豆 / 味噌汁</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>鮭とたまごの雑炊(小松菜を追加) / いちご</t>
-        </is>
-      </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>千切り野菜のだし豚しゃぶ / ご飯 / 冷凍ブロッコリー</t>
+          <t>厚揚げと大根の煮物 / ご飯 / ゆで卵</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>ブルーベリースムージー</t>
+          <t>白菜と豚肉の重ね蒸し / ご飯 / かぼちゃの煮物</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>ブルーベリー入りヨーグルト</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>10/16</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
           <t>金</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>ご飯 / ゆで卵 / 味噌汁</t>
-        </is>
-      </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>オムうどん</t>
+          <t>ご飯 / ゆで卵 / ヨーグルト+冷凍ブルーベリー</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>鯛の煮付け / ほうれん草のごま和え / ご飯</t>
+          <t>ひじきの煮物をのせたご飯 / けんちん汁</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>ヨーグルト+ブルーベリー</t>
+          <t>塩サバの味噌煮 / 冷凍ブロッコリー / ご飯 / 味噌汁</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>バナナ</t>
         </is>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
+          <t>10/17</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
           <t>土</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>トースト / 卵 / 牛乳</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>三色鶏そぼろ丼 / 味噌汁</t>
-        </is>
-      </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>肉豆腐 / 冷凍ブロッコリーのおかかバター / ご飯</t>
+          <t>豚汁 / おにぎり</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>バナナ</t>
+          <t>基本の親子丼 / 小松菜の煮浸し</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>ナッツ・牛乳</t>
         </is>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>10/18</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
           <t>日</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>簡単に(作り置きの仕込み)</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>惣菜・宅配も可</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>余り物で調整</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>ナッツ・牛乳</t>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>―</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>日曜に鶏の照り煮・おひたし・ゆで卵を作り置きし、ご飯を小分け冷凍する。ミルク併用でも授乳中なので量は本人の食欲に合わせる。</t>
+          <t>授乳中は妊娠前より約350kcal・たんぱく質約20gの上乗せが勧められる。ミルク併用でも量は本人の食欲に合わせる。作り置きは前日(日曜10/11)に調理。</t>
         </is>
       </c>
     </row>
@@ -718,395 +760,176 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>料理名</t>
+          <t>順</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>役割</t>
+          <t>品名</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>出典(デリッシュキッチン)</t>
+          <t>目安</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>使う日</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>メモ</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>卵と豆腐の味噌汁</t>
-        </is>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>汁物</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/372431553340376263</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>基本の親子丼</t>
-        </is>
+          <t>ご飯を炊いて小分け冷凍</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>約5合</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>毎食</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>最初に炊飯器をセット(提案)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>主食+主菜</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/197320405118092320</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>鯖の塩焼き</t>
-        </is>
+          <t>ひじきの煮物</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>約4人分</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>月夜・金昼</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>戻しながら他の作業を進める</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>主菜</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/197906490919486496</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>豚汁</t>
-        </is>
+          <t>かぼちゃの煮物</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>1/2個</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>月昼・木夜</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>レンジ版にすると時短</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>汁物(副菜兼用)</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/197484660219969894</t>
+          <t>小松菜と油揚げの煮浸し</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>約4人分</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>豚バラは脂が多いので豚こまに替えてもよい(提案)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>鮭とたまごの雑炊</t>
-        </is>
+          <t>火昼・水夜・土夜</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>レシピ記載は冷蔵3日・冷凍14日</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>主食+主菜</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/408107699302039880</t>
+          <t>ゆで卵</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>6個</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>小松菜を足すと鉄・葉酸が増える(提案)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>千切り野菜のだし豚しゃぶ</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>主菜+副菜</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/433714990541701537</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr"/>
+          <t>火朝・木昼・金朝ほか</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>―</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>オムうどん</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>主食+主菜</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/165433598944477587</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>冷凍うどん使用</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>鯛の煮付け</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>主菜</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/153237860613357862</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>ほうれん草のごま和え</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>副菜</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/134723216676487553</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>三色鶏そぼろ丼</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>主食+主菜</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/207028580079632788</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>肉豆腐</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>主菜</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/194111675098464660</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>リンクは牛肉。豚でも可</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>鶏ももと根菜の照り煮</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>主菜(日曜作り置き)</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/375619502815052886</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>月夜・水夜に使い回し</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>ほうれん草のおひたし</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>副菜(日曜作り置き)</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/390846387756991532</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2〜3日分を作り置き</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>冷凍ブロッコリーのおかかバター</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>副菜(レンジ)</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/328229145911755054</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>ブルーベリースムージー</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>間食・朝食</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/375479622474662329</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>補足リンク</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>冷凍ブロッコリーの解凍方法</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/419552908254642504</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>冷凍ブロッコリー活用レシピ19選</t>
-        </is>
-      </c>
-      <c r="C20" s="7" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/curations/7597</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>冷凍ブルーベリーレシピ</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/articles/31</t>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>所要時間の目安は1〜2時間(提案・未検証)。保存日数が記載されていない品は、早めに食べ切る。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId18"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1117,14 +940,538 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F47"/>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>料理名</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>役割</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>使う日</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>出典(デリッシュキッチン)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>メモ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ひじきの煮物</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>副菜(作り置き)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>月夜・金昼</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/200223304894645329</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>日曜に作る</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>小松菜と油揚げの煮浸し(作り置き向け)</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>副菜(作り置き)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>火昼・水夜・土夜</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/345087451330511890</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>元レシピは4人分。冷蔵3日・冷凍14日の目安が記載</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>かぼちゃの煮物</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>副菜(作り置き)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>月昼・木夜</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/186315122115871124</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>時短ならレンジ版(下記)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>かぼちゃの煮物(レンジ版)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>副菜(時短代替)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>―</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/134166380944556299</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>煮崩れしにくい</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>小松菜と油揚げの味噌汁</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>汁物</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>月朝</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/183853024563692671</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>豚の生姜焼き</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>主菜</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>月昼</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/551326352146433153</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>千切りキャベツを添える</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>鮭のちゃんちゃん焼き(フライパン)</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>主菜+副菜</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>月夜</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/313873402844676537</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>キャベツ・玉ねぎ・じゃがいも入り</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>けんちん汁</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>汁物(副菜兼用)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>火昼・金昼</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/145561470061511145</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>多めに作り翌日も</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>鶏の照り焼き(基本)</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>主菜</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>火夜・水昼</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/196290755478684070</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>残りで照り焼き丼</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>ブロッコリーとツナのマヨ和え</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>副菜</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>火夜</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/299398771979059613</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>冷凍は解凍後に水気を絞る</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>豆腐ハンバーグ(基本)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>主菜</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>水夜</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/196023942698239008</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>厚揚げと大根の煮物</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>主菜+副菜</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>木昼</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/357648074832609574</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>白菜と豚肉の重ね蒸し(レンジ)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>主菜+副菜</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>木夜</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/164138790271582611</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>加熱は肉に火が通るまで調整</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>塩サバの味噌煮</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>主菜</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>金夜</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/525069606923010402</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>豚汁</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>汁物</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>土昼</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/197484660219969894</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>豚バラは豚こまに替えてもよい(提案)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>基本の親子丼</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>主食+主菜</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>土夜</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/197320405118092320</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>補足リンク</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>冷凍ブロッコリーの解凍方法</t>
+        </is>
+      </c>
+      <c r="D20" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/419552908254642504</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>冷凍ブロッコリー活用レシピ19選</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/curations/7597</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>冷凍ブルーベリーレシピ</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/articles/31</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId19"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -1168,20 +1515,20 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>鶏もも肉</t>
+          <t>豚ロース(生姜焼き用)</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2</v>
+        <v>250</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>枚</t>
+          <t>g</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>照り煮・親子丼</t>
+          <t>生姜焼き</t>
         </is>
       </c>
       <c r="F2" s="8" t="n"/>
@@ -1194,11 +1541,11 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>鶏ひき肉</t>
+          <t>豚バラ薄切り(または豚こま)</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -1207,7 +1554,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>そぼろ丼</t>
+          <t>重ね蒸し・豚汁</t>
         </is>
       </c>
       <c r="F3" s="8" t="n"/>
@@ -1220,20 +1567,20 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>豚こま切れ</t>
+          <t>鶏もも肉</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>200</v>
+        <v>2</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>枚</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>豚汁・オムうどん</t>
+          <t>照り焼き・親子丼</t>
         </is>
       </c>
       <c r="F4" s="8" t="n"/>
@@ -1246,7 +1593,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>豚ロースしゃぶしゃぶ用</t>
+          <t>鶏ひき肉</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -1259,7 +1606,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>だし豚しゃぶ</t>
+          <t>豆腐ハンバーグ</t>
         </is>
       </c>
       <c r="F5" s="8" t="n"/>
@@ -1272,20 +1619,20 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>牛または豚の切り落とし</t>
+          <t>生鮭 切り身</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>150</v>
+        <v>2</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>切れ</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>肉豆腐</t>
+          <t>ちゃんちゃん焼き</t>
         </is>
       </c>
       <c r="F6" s="8" t="n"/>
@@ -1298,11 +1645,11 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>塩鮭 切り身</t>
+          <t>塩サバ</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -1311,7 +1658,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>おにぎり・雑炊ほか</t>
+          <t>味噌煮</t>
         </is>
       </c>
       <c r="F7" s="8" t="n"/>
@@ -1324,20 +1671,20 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>塩鯖</t>
+          <t>ツナ缶</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>切れ</t>
+          <t>缶</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>塩焼き</t>
+          <t>ブロッコリーのマヨ和え</t>
         </is>
       </c>
       <c r="F8" s="8" t="n"/>
@@ -1345,25 +1692,25 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>肉・魚</t>
+          <t>卵・大豆・乳</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>鯛などの白身魚 切り身</t>
+          <t>卵</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>切れ</t>
+          <t>個</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>煮付け</t>
+          <t>ゆで卵・親子丼・朝食</t>
         </is>
       </c>
       <c r="F9" s="8" t="n"/>
@@ -1376,20 +1723,20 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>卵</t>
+          <t>木綿豆腐</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>個</t>
+          <t>丁</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>ゆで卵・親子丼・雑炊ほか</t>
+          <t>豆腐ハンバーグ・けんちん汁</t>
         </is>
       </c>
       <c r="F10" s="8" t="n"/>
@@ -1402,11 +1749,11 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>絹豆腐</t>
+          <t>厚揚げ</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
@@ -1415,7 +1762,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>味噌汁・冷奴</t>
+          <t>煮物</t>
         </is>
       </c>
       <c r="F11" s="8" t="n"/>
@@ -1428,20 +1775,20 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>木綿豆腐</t>
+          <t>油揚げ</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>丁</t>
+          <t>枚</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>肉豆腐</t>
+          <t>煮浸し・味噌汁</t>
         </is>
       </c>
       <c r="F12" s="8" t="n"/>
@@ -1480,20 +1827,20 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>油揚げ</t>
+          <t>牛乳 1L</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>袋</t>
+          <t>本</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>味噌汁</t>
+          <t>朝食・間食</t>
         </is>
       </c>
       <c r="F14" s="8" t="n"/>
@@ -1506,7 +1853,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>牛乳 1L</t>
+          <t>無糖ヨーグルト 400g</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -1514,12 +1861,12 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>本</t>
+          <t>個</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>朝食・スムージー</t>
+          <t>朝食・間食</t>
         </is>
       </c>
       <c r="F15" s="8" t="n"/>
@@ -1532,20 +1879,20 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>無糖ヨーグルト 400g</t>
+          <t>スライスチーズ</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>個</t>
+          <t>袋</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>朝食・間食</t>
+          <t>朝食</t>
         </is>
       </c>
       <c r="F16" s="8" t="n"/>
@@ -1553,25 +1900,25 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>卵・大豆・乳</t>
+          <t>野菜</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>スライスチーズ</t>
+          <t>キャベツ</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>袋</t>
+          <t>個</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>朝食・間食</t>
+          <t>生姜焼き・ちゃんちゃん焼き</t>
         </is>
       </c>
       <c r="F17" s="8" t="n"/>
@@ -1584,20 +1931,20 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>大根</t>
+          <t>白菜</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>本</t>
+          <t>個</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>照り煮・豚汁</t>
+          <t>重ね蒸し(約5枚)</t>
         </is>
       </c>
       <c r="F18" s="8" t="n"/>
@@ -1610,7 +1957,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>にんじん</t>
+          <t>玉ねぎ</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
@@ -1618,12 +1965,12 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>本</t>
+          <t>個</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>照り煮・豚汁ほか</t>
+          <t>ちゃんちゃん焼きほか</t>
         </is>
       </c>
       <c r="F19" s="8" t="n"/>
@@ -1636,20 +1983,20 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>ごぼう</t>
+          <t>じゃがいも</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>本</t>
+          <t>個</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>豚汁</t>
+          <t>ちゃんちゃん焼き</t>
         </is>
       </c>
       <c r="F20" s="8" t="n"/>
@@ -1662,11 +2009,11 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>長ねぎ</t>
+          <t>にんじん</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
@@ -1675,7 +2022,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>豚汁ほか</t>
+          <t>ひじき・けんちん汁ほか</t>
         </is>
       </c>
       <c r="F21" s="8" t="n"/>
@@ -1688,20 +2035,20 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>玉ねぎ</t>
+          <t>大根</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>個</t>
+          <t>本</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>親子丼ほか</t>
+          <t>けんちん汁・煮物・重ね蒸し</t>
         </is>
       </c>
       <c r="F22" s="8" t="n"/>
@@ -1714,20 +2061,20 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>ほうれん草</t>
+          <t>ごぼう</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>袋</t>
+          <t>本</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>おひたし・ごま和え・そぼろ丼</t>
+          <t>けんちん汁・豚汁</t>
         </is>
       </c>
       <c r="F23" s="8" t="n"/>
@@ -1740,20 +2087,20 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>小松菜</t>
+          <t>長ねぎ</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>袋</t>
+          <t>本</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>雑炊</t>
+          <t>重ね蒸しほか</t>
         </is>
       </c>
       <c r="F24" s="8" t="n"/>
@@ -1766,20 +2113,20 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>キャベツ</t>
+          <t>小松菜</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>0.25</v>
+        <v>2</v>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>個</t>
+          <t>束</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>だし豚しゃぶ</t>
+          <t>煮浸し・味噌汁</t>
         </is>
       </c>
       <c r="F25" s="8" t="n"/>
@@ -1792,20 +2139,20 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>もやし</t>
+          <t>かぼちゃ</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>袋</t>
+          <t>個</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>オムうどん</t>
+          <t>煮物</t>
         </is>
       </c>
       <c r="F26" s="8" t="n"/>
@@ -1818,7 +2165,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>しょうが・絹さや</t>
+          <t>こんにゃく</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
@@ -1826,12 +2173,12 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>式</t>
+          <t>枚</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>照り煮・煮付け</t>
+          <t>けんちん汁・豚汁</t>
         </is>
       </c>
       <c r="F27" s="8" t="n"/>
@@ -1844,7 +2191,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>こんにゃく</t>
+          <t>しょうが</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -1852,12 +2199,12 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>枚</t>
+          <t>かけ</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>豚汁</t>
+          <t>生姜焼き</t>
         </is>
       </c>
       <c r="F28" s="8" t="n"/>
@@ -1883,7 +2230,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>副菜(150g×約3回)</t>
+          <t>副菜</t>
         </is>
       </c>
       <c r="F29" s="8" t="n"/>
@@ -1909,7 +2256,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>ヨーグルト・スムージー</t>
+          <t>朝食・間食</t>
         </is>
       </c>
       <c r="F30" s="8" t="n"/>
@@ -1922,20 +2269,20 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>冷凍うどん</t>
+          <t>乾燥ひじき</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>玉</t>
+          <t>袋</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>オムうどん</t>
+          <t>ひじきの煮物(20g)</t>
         </is>
       </c>
       <c r="F31" s="8" t="n"/>
@@ -1974,20 +2321,20 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>キウイ</t>
+          <t>バナナ</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>個</t>
+          <t>房</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>朝食</t>
+          <t>朝食・間食</t>
         </is>
       </c>
       <c r="F33" s="8" t="n"/>
@@ -2000,20 +2347,20 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>みかん</t>
+          <t>キウイ</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>袋</t>
+          <t>個</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>昼</t>
+          <t>ビタミンC補給</t>
         </is>
       </c>
       <c r="F34" s="8" t="n"/>
@@ -2026,7 +2373,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>いちご</t>
+          <t>みかん</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2034,12 +2381,12 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>パック</t>
+          <t>袋</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>昼</t>
+          <t>ビタミンC補給</t>
         </is>
       </c>
       <c r="F35" s="8" t="n"/>
@@ -2047,25 +2394,25 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>果物</t>
+          <t>主食</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>バナナ</t>
+          <t>米</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>房</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>朝食・間食</t>
+          <t>毎食</t>
         </is>
       </c>
       <c r="F36" s="8" t="n"/>
@@ -2078,20 +2425,20 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>米</t>
+          <t>食パン</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>袋</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>毎食</t>
+          <t>朝食</t>
         </is>
       </c>
       <c r="F37" s="8" t="n"/>
@@ -2104,7 +2451,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>食パン</t>
+          <t>焼きのり</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
@@ -2117,7 +2464,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>朝食</t>
+          <t>おにぎり</t>
         </is>
       </c>
       <c r="F38" s="8" t="n"/>
@@ -2125,12 +2472,12 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>調味料</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>焼きのり</t>
+          <t>味噌・顆粒だし・しょうゆ・みりん・酒・砂糖・塩</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
@@ -2138,12 +2485,12 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>袋</t>
+          <t>式</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>おにぎり</t>
+          <t>在庫を確認</t>
         </is>
       </c>
       <c r="F39" s="8" t="n"/>
@@ -2156,7 +2503,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>味噌・顆粒だし・しょうゆ・みりん・酒・砂糖・塩</t>
+          <t>めんつゆ・ポン酢・バター・薄力粉・マヨネーズ・鶏ガラスープの素・ごま油</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
@@ -2174,67 +2521,41 @@
       </c>
       <c r="F40" s="8" t="n"/>
     </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>調味料</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>白すりごま・かつお節・めんつゆ・ポン酢・バター・お好み焼きソース</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>式</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>在庫を確認</t>
-        </is>
-      </c>
-      <c r="F41" s="8" t="n"/>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>品目数</t>
+        </is>
+      </c>
+      <c r="B42" s="6">
+        <f>COUNTA(B2:B40)</f>
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>品目数</t>
+          <t>購入済</t>
         </is>
       </c>
       <c r="B43" s="6">
-        <f>COUNTA(B2:B41)</f>
+        <f>COUNTIF(F2:F40,"○")</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>購入済</t>
+          <t>残り</t>
         </is>
       </c>
       <c r="B44" s="6">
-        <f>COUNTIF(F2:F41,"○")</f>
+        <f>B42-B43</f>
         <v/>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>残り</t>
-        </is>
-      </c>
-      <c r="B45" s="6">
-        <f>B43-B44</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="3" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>数量は2人分の概算(Claudeの推定)。在庫を差し引いて調整。F列に○を入れると集計される。</t>
         </is>
@@ -2245,7 +2566,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2276,7 +2597,7 @@
           <t>主食+主菜+副菜をそろえると栄養がととのいやすい</t>
         </is>
       </c>
-      <c r="B2" s="9" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>https://www.city.bunkyo.lg.jp/documents/1540/2024321215312.pdf</t>
         </is>
@@ -2288,7 +2609,7 @@
           <t>授乳中は妊娠前より約350kcal・たんぱく質約20gの上乗せが勧められる</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>https://www.med.jrc.or.jp/Portals/0/resources/hospital/clinic/sanka/eiyo.pdf</t>
         </is>
@@ -2300,7 +2621,7 @@
           <t>鉄はビタミンCと一緒に。和食中心・脂っこい物と菓子は控えめ・水分補給</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>https://www.kenko-shokuiku.city.nagoya.jp/pdf/ninsanpu_syokuji.pdf</t>
         </is>
@@ -2312,7 +2633,7 @@
           <t>日本人の食事摂取基準(2025年版)公式</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>https://www.mhlw.go.jp/content/10904750/001542297.pdf</t>
         </is>
@@ -2324,7 +2645,7 @@
           <t>冷凍野菜の栄養(生より少ないビタミンCもある)</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>https://hugkum.sho.jp/402470</t>
         </is>

</xml_diff>

<commit_message>
Use chicken breast for teriyaki; update recipe and shopping list
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016abfmfMm3FJdNo4xsxKHTV
</commit_message>
<xml_diff>
--- a/献立表_レシピ_買い物リスト.xlsx
+++ b/献立表_レシピ_買い物リスト.xlsx
@@ -573,7 +573,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>鶏の照り焼き / ブロッコリーとツナのマヨ和え / ご飯</t>
+          <t>鶏むねの照り焼き / ブロッコリーとツナのマヨ和え / ご飯</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1192,7 +1192,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>鶏の照り焼き(基本)</t>
+          <t>鶏むねの照り焼き(冷めても柔らか)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1207,12 +1207,12 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>https://delishkitchen.tv/recipes/196290755478684070</t>
+          <t>https://delishkitchen.tv/recipes/118520140160565572</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>残りで照り焼き丼</t>
+          <t>鶏むね肉を使用。残りで水昼の照り焼き丼</t>
         </is>
       </c>
     </row>
@@ -1389,6 +1389,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr"/>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
@@ -1571,7 +1572,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -1580,7 +1581,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>照り焼き・親子丼</t>
+          <t>親子丼</t>
         </is>
       </c>
       <c r="F4" s="8" t="n"/>
@@ -2521,6 +2522,36 @@
       </c>
       <c r="F40" s="8" t="n"/>
     </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>肉・魚</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>鶏むね肉</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>枚</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>照り焼き(火夜)・照り焼き丼(水昼)</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
@@ -2528,7 +2559,7 @@
         </is>
       </c>
       <c r="B42" s="6">
-        <f>COUNTA(B2:B40)</f>
+        <f>COUNTA(B2:B41)</f>
         <v/>
       </c>
     </row>
@@ -2539,7 +2570,7 @@
         </is>
       </c>
       <c r="B43" s="6">
-        <f>COUNTIF(F2:F40,"○")</f>
+        <f>COUNTIF(F2:F41,"○")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update workbook for week of 10/19
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016abfmfMm3FJdNo4xsxKHTV
</commit_message>
<xml_diff>
--- a/献立表_レシピ_買い物リスト.xlsx
+++ b/献立表_レシピ_買い物リスト.xlsx
@@ -521,7 +521,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>10/12</t>
+          <t>10/19</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -531,17 +531,17 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>ご飯 / 小松菜と油揚げの味噌汁 / 納豆</t>
+          <t>ご飯 / さつまいもと厚揚げの味噌汁 / 納豆</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>豚の生姜焼き+千切りキャベツ / ご飯 / かぼちゃの煮物</t>
+          <t>蒸し鶏+冷凍ブロッコリー / ご飯</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>鮭のちゃんちゃん焼き / ご飯 / ひじきの煮物</t>
+          <t>肉じゃが / ほうれん草と卵のソテー / ご飯</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -553,7 +553,7 @@
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>10/13</t>
+          <t>10/20</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -563,17 +563,17 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>ご飯 / ゆで卵 / ヨーグルト+冷凍ブルーベリー</t>
+          <t>トースト / ヨーグルト+冷凍ブルーベリー / バナナ</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>けんちん汁 / おにぎり / 小松菜の煮浸し</t>
+          <t>筑前煮 / ご飯 / 味噌汁</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>鶏むねの照り焼き / ブロッコリーとツナのマヨ和え / ご飯</t>
+          <t>タラのムニエル / 冷凍ブロッコリー / ご飯 / 味噌汁</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -585,7 +585,7 @@
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>10/14</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -595,17 +595,17 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>トースト / チーズ / バナナ / 牛乳</t>
+          <t>ご飯 / ゆで卵 / 白菜とさつまいもの味噌汁</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>照り焼き丼(残り) / 味噌汁</t>
+          <t>カオマンガイ風 蒸し鶏ごはん</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>豆腐ハンバーグ / 小松菜の煮浸し / ご飯</t>
+          <t>鶏肉とほうれん草のクリームシチュー / パン</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>10/15</t>
+          <t>10/22</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -627,29 +627,29 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>ご飯 / 納豆 / 味噌汁</t>
+          <t>トースト / チーズ / 牛乳 / バナナ</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>厚揚げと大根の煮物 / ご飯 / ゆで卵</t>
+          <t>シチューの残り / ご飯</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>白菜と豚肉の重ね蒸し / ご飯 / かぼちゃの煮物</t>
+          <t>鮭としめじの炊き込みごはん / 味噌汁 / ほうれん草のおひたし</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>ブルーベリー入りヨーグルト</t>
+          <t>ヨーグルト+ブルーベリー</t>
         </is>
       </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>10/16</t>
+          <t>10/23</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -659,17 +659,17 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>ご飯 / ゆで卵 / ヨーグルト+冷凍ブルーベリー</t>
+          <t>炊き込みご飯の残り / ゆで卵</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>ひじきの煮物をのせたご飯 / けんちん汁</t>
+          <t>肉じゃがの残り / ご飯</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>塩サバの味噌煮 / 冷凍ブロッコリー / ご飯 / 味噌汁</t>
+          <t>肉豆腐 / 冷凍ブロッコリー / ご飯</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -681,7 +681,7 @@
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>10/17</t>
+          <t>10/24</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -696,12 +696,12 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>豚汁 / おにぎり</t>
+          <t>豚肉とさつまいもの味噌汁 / おにぎり</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>基本の親子丼 / 小松菜の煮浸し</t>
+          <t>塩サバの味噌煮 / ご飯 / 味噌汁</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -713,7 +713,7 @@
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>10/18</t>
+          <t>10/25</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -745,7 +745,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>授乳中は妊娠前より約350kcal・たんぱく質約20gの上乗せが勧められる。ミルク併用でも量は本人の食欲に合わせる。作り置きは前日(日曜10/11)に調理。</t>
+          <t>授乳中は妊娠前より約350kcal・たんぱく質約20gの上乗せが勧められる。ミルク併用でも量は本人の食欲に合わせる。作り置きは前日(日曜10/18)に調理。</t>
         </is>
       </c>
     </row>
@@ -828,7 +828,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>ひじきの煮物</t>
+          <t>筑前煮</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -838,12 +838,12 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>月夜・金昼</t>
+          <t>火昼</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>戻しながら他の作業を進める</t>
+          <t>干ししいたけは前日に戻しておく(戻し汁を使う)</t>
         </is>
       </c>
     </row>
@@ -853,22 +853,22 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>かぼちゃの煮物</t>
+          <t>蒸し鶏(生姜風味・レンジ)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>1/2個</t>
+          <t>むね肉1枚</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>月昼・木夜</t>
+          <t>月昼・水昼</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>レンジ版にすると時短</t>
+          <t>レンジ加熱後、粗熱を取って保存</t>
         </is>
       </c>
     </row>
@@ -878,45 +878,20 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>小松菜と油揚げの煮浸し</t>
+          <t>ゆで卵</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>約4人分</t>
+          <t>6個</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>火昼・水夜・土夜</t>
+          <t>水朝・金朝ほか</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>レシピ記載は冷蔵3日・冷凍14日</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>ゆで卵</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>6個</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>火朝・木昼・金朝ほか</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>―</t>
         </is>
@@ -940,7 +915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -980,130 +955,126 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ひじきの煮物</t>
+          <t>筑前煮</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>副菜(作り置き)</t>
+          <t>主菜+副菜(作り置き)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>月夜・金昼</t>
+          <t>火昼</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>https://delishkitchen.tv/recipes/200223304894645329</t>
+          <t>https://delishkitchen.tv/recipes/202971540197736870</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>日曜に作る</t>
+          <t>日曜に作る。干ししいたけの戻し汁を煮汁に使う</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>小松菜と油揚げの煮浸し(作り置き向け)</t>
+          <t>蒸し鶏(生姜風味・レンジ)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>副菜(作り置き)</t>
+          <t>主菜(作り置き)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>火昼・水夜・土夜</t>
+          <t>月昼・水昼</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>https://delishkitchen.tv/recipes/345087451330511890</t>
+          <t>https://delishkitchen.tv/recipes/149665586794725670</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>元レシピは4人分。冷蔵3日・冷凍14日の目安が記載</t>
+          <t>鶏むね肉を使用</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>かぼちゃの煮物</t>
+          <t>さつまいもと厚揚げの味噌汁</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>副菜(作り置き)</t>
+          <t>汁物</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>月昼・木夜</t>
+          <t>月朝</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>https://delishkitchen.tv/recipes/186315122115871124</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>時短ならレンジ版(下記)</t>
-        </is>
-      </c>
+          <t>https://delishkitchen.tv/recipes/379110584001496297</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>かぼちゃの煮物(レンジ版)</t>
+          <t>肉じゃが(基本)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>副菜(時短代替)</t>
+          <t>主菜+副菜</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>―</t>
+          <t>月夜・金昼</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>https://delishkitchen.tv/recipes/134166380944556299</t>
+          <t>https://delishkitchen.tv/recipes/153240773708480781</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>煮崩れしにくい</t>
+          <t>残りを翌昼に回す</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>小松菜と油揚げの味噌汁</t>
+          <t>ほうれん草と卵のソテー</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>汁物</t>
+          <t>副菜</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>月朝</t>
+          <t>月夜</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>https://delishkitchen.tv/recipes/183853024563692671</t>
+          <t>https://delishkitchen.tv/recipes/337352711349470342</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -1111,7 +1082,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>豚の生姜焼き</t>
+          <t>タラのムニエル</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -1121,147 +1092,139 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>月昼</t>
+          <t>火夜</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>https://delishkitchen.tv/recipes/551326352146433153</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>千切りキャベツを添える</t>
-        </is>
-      </c>
+          <t>https://delishkitchen.tv/recipes/357472571177829394</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>鮭のちゃんちゃん焼き(フライパン)</t>
+          <t>白菜とさつまいもの味噌汁</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>主菜+副菜</t>
+          <t>汁物</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>月夜</t>
+          <t>水朝</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>https://delishkitchen.tv/recipes/313873402844676537</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>キャベツ・玉ねぎ・じゃがいも入り</t>
-        </is>
-      </c>
+          <t>https://delishkitchen.tv/recipes/173108175090745836</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>けんちん汁</t>
+          <t>カオマンガイ風 蒸し鶏ごはん</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>汁物(副菜兼用)</t>
+          <t>主食+主菜</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>火昼・金昼</t>
+          <t>水昼</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>https://delishkitchen.tv/recipes/145561470061511145</t>
+          <t>https://delishkitchen.tv/recipes/292861887203246397</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>多めに作り翌日も</t>
+          <t>作り置きの蒸し鶏を使う</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>鶏むねの照り焼き(冷めても柔らか)</t>
+          <t>鶏肉とほうれん草のクリームシチュー</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>主菜</t>
+          <t>主菜+副菜</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>火夜・水昼</t>
+          <t>水夜・木昼</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>https://delishkitchen.tv/recipes/118520140160565572</t>
+          <t>https://delishkitchen.tv/recipes/329056906922427410</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>鶏むね肉を使用。残りで水昼の照り焼き丼</t>
+          <t>残りを翌昼に回す</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>ブロッコリーとツナのマヨ和え</t>
+          <t>鮭としめじの炊き込みごはん</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>副菜</t>
+          <t>主食+主菜</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>火夜</t>
+          <t>木夜・金朝</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>https://delishkitchen.tv/recipes/299398771979059613</t>
+          <t>https://delishkitchen.tv/recipes/139805641278488995</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>冷凍は解凍後に水気を絞る</t>
+          <t>残りを翌朝に回す</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>豆腐ハンバーグ(基本)</t>
+          <t>ほうれん草のおひたし</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>主菜</t>
+          <t>副菜</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>水夜</t>
+          <t>木夜</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>https://delishkitchen.tv/recipes/196023942698239008</t>
+          <t>https://delishkitchen.tv/recipes/390846387756991532</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
@@ -1269,52 +1232,52 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>厚揚げと大根の煮物</t>
+          <t>肉豆腐</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>主菜+副菜</t>
+          <t>主菜</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>木昼</t>
+          <t>金夜</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>https://delishkitchen.tv/recipes/357648074832609574</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
+          <t>https://delishkitchen.tv/recipes/194111675098464660</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>リンクは牛肉。豚でも可</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>白菜と豚肉の重ね蒸し(レンジ)</t>
+          <t>豚肉とさつまいもの味噌汁</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>主菜+副菜</t>
+          <t>汁物</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>木夜</t>
+          <t>土昼</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>https://delishkitchen.tv/recipes/164138790271582611</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>加熱は肉に火が通るまで調整</t>
-        </is>
-      </c>
+          <t>https://delishkitchen.tv/recipes/180204471723229588</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1329,7 +1292,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>金夜</t>
+          <t>土夜</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1339,95 +1302,44 @@
       </c>
       <c r="E15" s="2" t="inlineStr"/>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>豚汁</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>汁物</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>土昼</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/197484660219969894</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>豚バラは豚こまに替えてもよい(提案)</t>
-        </is>
-      </c>
-    </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>基本の親子丼</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>主食+主菜</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>土夜</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/197320405118092320</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr"/>
-    </row>
-    <row r="18"/>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>補足リンク</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>冷凍ブロッコリーの解凍方法</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/419552908254642504</t>
+        </is>
+      </c>
+    </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>補足リンク</t>
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>冷凍ブロッコリー活用レシピ19選</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/curations/7597</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>冷凍ブロッコリーの解凍方法</t>
+          <t>冷凍ブルーベリーレシピ</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/419552908254642504</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>冷凍ブロッコリー活用レシピ19選</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/curations/7597</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>冷凍ブルーベリーレシピ</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
         <is>
           <t>https://delishkitchen.tv/articles/31</t>
         </is>
@@ -1449,11 +1361,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1465,7 +1375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1516,20 +1426,20 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>豚ロース(生姜焼き用)</t>
+          <t>鶏むね肉</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>250</v>
+        <v>1</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>枚</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>生姜焼き</t>
+          <t>蒸し鶏</t>
         </is>
       </c>
       <c r="F2" s="8" t="n"/>
@@ -1542,20 +1452,20 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>豚バラ薄切り(または豚こま)</t>
+          <t>鶏もも肉</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>300</v>
+        <v>2</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>枚</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>重ね蒸し・豚汁</t>
+          <t>筑前煮・クリームシチュー</t>
         </is>
       </c>
       <c r="F3" s="8" t="n"/>
@@ -1568,20 +1478,20 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>鶏もも肉</t>
+          <t>牛または豚の切り落とし</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>1</v>
+        <v>350</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>枚</t>
+          <t>g</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>親子丼</t>
+          <t>肉じゃが・肉豆腐</t>
         </is>
       </c>
       <c r="F4" s="8" t="n"/>
@@ -1594,11 +1504,11 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>鶏ひき肉</t>
+          <t>豚こま切れ</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -1607,7 +1517,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>豆腐ハンバーグ</t>
+          <t>豚肉とさつまいもの味噌汁</t>
         </is>
       </c>
       <c r="F5" s="8" t="n"/>
@@ -1620,7 +1530,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>生鮭 切り身</t>
+          <t>タラ 切り身</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -1633,7 +1543,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>ちゃんちゃん焼き</t>
+          <t>ムニエル</t>
         </is>
       </c>
       <c r="F6" s="8" t="n"/>
@@ -1646,7 +1556,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>塩サバ</t>
+          <t>生鮭 切り身</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -1659,7 +1569,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>味噌煮</t>
+          <t>炊き込みごはん</t>
         </is>
       </c>
       <c r="F7" s="8" t="n"/>
@@ -1672,20 +1582,20 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>ツナ缶</t>
+          <t>塩サバ</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>缶</t>
+          <t>切れ</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>ブロッコリーのマヨ和え</t>
+          <t>味噌煮</t>
         </is>
       </c>
       <c r="F8" s="8" t="n"/>
@@ -1702,7 +1612,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -1711,7 +1621,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>ゆで卵・親子丼・朝食</t>
+          <t>ゆで卵・ソテー・朝食</t>
         </is>
       </c>
       <c r="F9" s="8" t="n"/>
@@ -1728,7 +1638,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -1737,7 +1647,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>豆腐ハンバーグ・けんちん汁</t>
+          <t>肉豆腐</t>
         </is>
       </c>
       <c r="F10" s="8" t="n"/>
@@ -1763,7 +1673,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>煮物</t>
+          <t>味噌汁</t>
         </is>
       </c>
       <c r="F11" s="8" t="n"/>
@@ -1776,20 +1686,20 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>油揚げ</t>
+          <t>納豆</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>枚</t>
+          <t>パック</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>煮浸し・味噌汁</t>
+          <t>朝食</t>
         </is>
       </c>
       <c r="F12" s="8" t="n"/>
@@ -1802,20 +1712,20 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>納豆</t>
+          <t>牛乳 1L</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>パック</t>
+          <t>本</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>朝食</t>
+          <t>シチュー・朝食</t>
         </is>
       </c>
       <c r="F13" s="8" t="n"/>
@@ -1828,15 +1738,15 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>牛乳 1L</t>
+          <t>無糖ヨーグルト 400g</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>本</t>
+          <t>個</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1854,15 +1764,15 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>無糖ヨーグルト 400g</t>
+          <t>スライスチーズ</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>個</t>
+          <t>袋</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1875,25 +1785,25 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>卵・大豆・乳</t>
+          <t>野菜</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>スライスチーズ</t>
+          <t>じゃがいも</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>袋</t>
+          <t>個</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>朝食</t>
+          <t>肉じゃが・シチュー</t>
         </is>
       </c>
       <c r="F16" s="8" t="n"/>
@@ -1906,20 +1816,20 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>キャベツ</t>
+          <t>にんじん</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.5</v>
+        <v>3</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>個</t>
+          <t>本</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>生姜焼き・ちゃんちゃん焼き</t>
+          <t>肉じゃが・筑前煮・シチュー</t>
         </is>
       </c>
       <c r="F17" s="8" t="n"/>
@@ -1932,11 +1842,11 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>白菜</t>
+          <t>玉ねぎ</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0.25</v>
+        <v>3</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
@@ -1945,7 +1855,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>重ね蒸し(約5枚)</t>
+          <t>肉じゃがほか</t>
         </is>
       </c>
       <c r="F18" s="8" t="n"/>
@@ -1958,20 +1868,20 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>玉ねぎ</t>
+          <t>さつまいも</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>個</t>
+          <t>本</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>ちゃんちゃん焼きほか</t>
+          <t>味噌汁</t>
         </is>
       </c>
       <c r="F19" s="8" t="n"/>
@@ -1984,11 +1894,11 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>じゃがいも</t>
+          <t>白菜</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>2</v>
+        <v>0.25</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -1997,7 +1907,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>ちゃんちゃん焼き</t>
+          <t>味噌汁</t>
         </is>
       </c>
       <c r="F20" s="8" t="n"/>
@@ -2010,7 +1920,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>にんじん</t>
+          <t>ほうれん草</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -2018,12 +1928,12 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>本</t>
+          <t>袋</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>ひじき・けんちん汁ほか</t>
+          <t>ソテー・シチュー・おひたし</t>
         </is>
       </c>
       <c r="F21" s="8" t="n"/>
@@ -2036,7 +1946,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>大根</t>
+          <t>ごぼう</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -2049,7 +1959,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>けんちん汁・煮物・重ね蒸し</t>
+          <t>筑前煮</t>
         </is>
       </c>
       <c r="F22" s="8" t="n"/>
@@ -2062,7 +1972,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>ごぼう</t>
+          <t>れんこん</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -2070,12 +1980,12 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>本</t>
+          <t>節</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>けんちん汁・豚汁</t>
+          <t>筑前煮</t>
         </is>
       </c>
       <c r="F23" s="8" t="n"/>
@@ -2088,20 +1998,20 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>長ねぎ</t>
+          <t>里芋</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>本</t>
+          <t>個</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>重ね蒸しほか</t>
+          <t>筑前煮</t>
         </is>
       </c>
       <c r="F24" s="8" t="n"/>
@@ -2114,20 +2024,20 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>小松菜</t>
+          <t>こんにゃく</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>束</t>
+          <t>枚</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>煮浸し・味噌汁</t>
+          <t>筑前煮</t>
         </is>
       </c>
       <c r="F25" s="8" t="n"/>
@@ -2140,20 +2050,20 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>かぼちゃ</t>
+          <t>長ねぎ</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>個</t>
+          <t>本</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>煮物</t>
+          <t>肉豆腐・蒸し鶏ごはん</t>
         </is>
       </c>
       <c r="F26" s="8" t="n"/>
@@ -2166,20 +2076,20 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>こんにゃく</t>
+          <t>しめじ</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>枚</t>
+          <t>パック</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>けんちん汁・豚汁</t>
+          <t>炊き込みごはん・シチュー</t>
         </is>
       </c>
       <c r="F27" s="8" t="n"/>
@@ -2192,7 +2102,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>しょうが</t>
+          <t>いんげん</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2200,12 +2110,12 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>かけ</t>
+          <t>袋</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>生姜焼き</t>
+          <t>肉じゃが</t>
         </is>
       </c>
       <c r="F28" s="8" t="n"/>
@@ -2270,20 +2180,20 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>乾燥ひじき</t>
+          <t>干ししいたけ</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>袋</t>
+          <t>個</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>ひじきの煮物(20g)</t>
+          <t>筑前煮</t>
         </is>
       </c>
       <c r="F31" s="8" t="n"/>
@@ -2291,12 +2201,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>冷凍・乾物</t>
+          <t>果物</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>乾燥わかめ</t>
+          <t>バナナ</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2304,12 +2214,12 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>袋</t>
+          <t>房</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>味噌汁</t>
+          <t>朝食・間食</t>
         </is>
       </c>
       <c r="F32" s="8" t="n"/>
@@ -2317,25 +2227,25 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>果物</t>
+          <t>主食</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>バナナ</t>
+          <t>米</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>房</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>朝食・間食</t>
+          <t>毎食</t>
         </is>
       </c>
       <c r="F33" s="8" t="n"/>
@@ -2343,25 +2253,25 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>果物</t>
+          <t>主食</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>キウイ</t>
+          <t>食パン</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>個</t>
+          <t>袋</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>ビタミンC補給</t>
+          <t>朝食・夕食</t>
         </is>
       </c>
       <c r="F34" s="8" t="n"/>
@@ -2369,12 +2279,12 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>果物</t>
+          <t>主食</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>みかん</t>
+          <t>焼きのり</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
@@ -2387,7 +2297,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>ビタミンC補給</t>
+          <t>おにぎり</t>
         </is>
       </c>
       <c r="F35" s="8" t="n"/>
@@ -2395,25 +2305,25 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>調味料</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>米</t>
+          <t>味噌・顆粒だし・しょうゆ・みりん・酒・砂糖・塩こしょう</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>式</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>毎食</t>
+          <t>在庫を確認</t>
         </is>
       </c>
       <c r="F36" s="8" t="n"/>
@@ -2421,12 +2331,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>調味料</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>食パン</t>
+          <t>薄力粉・バター・オリーブオイル・しょうが</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
@@ -2434,159 +2344,51 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>袋</t>
+          <t>式</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>朝食</t>
+          <t>在庫を確認</t>
         </is>
       </c>
       <c r="F37" s="8" t="n"/>
     </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>主食</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>焼きのり</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>袋</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>おにぎり</t>
-        </is>
-      </c>
-      <c r="F38" s="8" t="n"/>
-    </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>調味料</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>味噌・顆粒だし・しょうゆ・みりん・酒・砂糖・塩</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>式</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>在庫を確認</t>
-        </is>
-      </c>
-      <c r="F39" s="8" t="n"/>
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>品目数</t>
+        </is>
+      </c>
+      <c r="B39" s="6">
+        <f>COUNTA(B2:B37)</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>調味料</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>めんつゆ・ポン酢・バター・薄力粉・マヨネーズ・鶏ガラスープの素・ごま油</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>式</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>在庫を確認</t>
-        </is>
-      </c>
-      <c r="F40" s="8" t="n"/>
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>購入済</t>
+        </is>
+      </c>
+      <c r="B40" s="6">
+        <f>COUNTIF(F2:F37,"○")</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>肉・魚</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>鶏むね肉</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>枚</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>照り焼き(火夜)・照り焼き丼(水昼)</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>品目数</t>
-        </is>
-      </c>
-      <c r="B42" s="6">
-        <f>COUNTA(B2:B41)</f>
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>残り</t>
+        </is>
+      </c>
+      <c r="B41" s="6">
+        <f>B39-B40</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>購入済</t>
-        </is>
-      </c>
-      <c r="B43" s="6">
-        <f>COUNTIF(F2:F41,"○")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>残り</t>
-        </is>
-      </c>
-      <c r="B44" s="6">
-        <f>B42-B43</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="3" t="inlineStr">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>数量は2人分の概算(Claudeの推定)。在庫を差し引いて調整。F列に○を入れると集計される。</t>
         </is>

</xml_diff>

<commit_message>
Set current week to 10/16-10/22 and add next week plan
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016abfmfMm3FJdNo4xsxKHTV
</commit_message>
<xml_diff>
--- a/献立表_レシピ_買い物リスト.xlsx
+++ b/献立表_レシピ_買い物リスト.xlsx
@@ -7,11 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="献立表" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="作り置き" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="レシピ" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="買い物リスト" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="出典・基礎原理" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="今週_献立" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="今週_作り置き" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="今週_買い物" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="来週_献立" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="来週_作り置き" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="来週_買い物" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="レシピ" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="出典・基礎原理" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -45,14 +48,14 @@
     </font>
     <font>
       <name val="Meiryo"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Meiryo"/>
       <color rgb="000563C1"/>
       <sz val="10"/>
       <u val="single"/>
-    </font>
-    <font>
-      <name val="Meiryo"/>
-      <b val="1"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -103,13 +106,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -521,12 +524,12 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>10/19</t>
+          <t>10/16</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>月</t>
+          <t>金</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -553,12 +556,12 @@
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>10/20</t>
+          <t>10/17</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>火</t>
+          <t>土</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -585,12 +588,12 @@
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>10/21</t>
+          <t>10/18</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>水</t>
+          <t>日</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -617,12 +620,12 @@
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>10/22</t>
+          <t>10/19</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>木</t>
+          <t>月</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -649,12 +652,12 @@
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>10/23</t>
+          <t>10/20</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>金</t>
+          <t>火</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -681,12 +684,12 @@
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>10/24</t>
+          <t>10/21</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>土</t>
+          <t>水</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -713,12 +716,12 @@
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>10/25</t>
+          <t>10/22</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>日</t>
+          <t>木</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -745,7 +748,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>授乳中は妊娠前より約350kcal・たんぱく質約20gの上乗せが勧められる。ミルク併用でも量は本人の食欲に合わせる。作り置きは前日(日曜10/18)に調理。</t>
+          <t>今週=10/16(金)〜10/22(木)。授乳中は妊娠前より約350kcal・たんぱく質約20gの上乗せが勧められる。ミルク併用でも量は本人の食欲に合わせる。作り置きは今日10/15(木)。</t>
         </is>
       </c>
     </row>
@@ -838,7 +841,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>火昼</t>
+          <t>土昼</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -863,7 +866,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>月昼・水昼</t>
+          <t>金昼・日昼</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -888,7 +891,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>水朝・金朝ほか</t>
+          <t>日朝・火朝ほか</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -900,7 +903,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>所要時間の目安は1〜2時間(提案・未検証)。保存日数が記載されていない品は、早めに食べ切る。</t>
+          <t>保存日数が記載されていない品は早めに食べ切る。</t>
         </is>
       </c>
     </row>
@@ -915,456 +918,1026 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>料理名</t>
+          <t>区分</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>役割</t>
+          <t>品名</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>使う日</t>
+          <t>数量</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>出典(デリッシュキッチン)</t>
+          <t>単位</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>メモ</t>
+          <t>用途</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>購入済(○)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>筑前煮</t>
+          <t>肉・魚</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>主菜+副菜(作り置き)</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>火昼</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/202971540197736870</t>
+          <t>鶏むね肉</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>枚</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>日曜に作る。干ししいたけの戻し汁を煮汁に使う</t>
-        </is>
-      </c>
+          <t>蒸し鶏</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>蒸し鶏(生姜風味・レンジ)</t>
+          <t>肉・魚</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>主菜(作り置き)</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>月昼・水昼</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/149665586794725670</t>
+          <t>鶏もも肉</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>枚</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>鶏むね肉を使用</t>
-        </is>
-      </c>
+          <t>筑前煮・クリームシチュー</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>さつまいもと厚揚げの味噌汁</t>
+          <t>肉・魚</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>汁物</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>月朝</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/379110584001496297</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr"/>
+          <t>牛または豚の切り落とし</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>350</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>肉じゃが・肉豆腐</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>肉じゃが(基本)</t>
+          <t>肉・魚</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>主菜+副菜</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>月夜・金昼</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/153240773708480781</t>
+          <t>豚こま切れ</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>g</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>残りを翌昼に回す</t>
-        </is>
-      </c>
+          <t>豚肉とさつまいもの味噌汁</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ほうれん草と卵のソテー</t>
+          <t>肉・魚</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>副菜</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>月夜</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/337352711349470342</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
+          <t>タラ 切り身</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>切れ</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>ムニエル</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>タラのムニエル</t>
+          <t>肉・魚</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>主菜</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>火夜</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/357472571177829394</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
+          <t>生鮭 切り身</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>切れ</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>炊き込みごはん</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>白菜とさつまいもの味噌汁</t>
+          <t>肉・魚</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>汁物</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>水朝</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/173108175090745836</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
+          <t>塩サバ</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>切れ</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>味噌煮</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>カオマンガイ風 蒸し鶏ごはん</t>
+          <t>卵・大豆・乳</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>主食+主菜</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>水昼</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/292861887203246397</t>
+          <t>卵</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>個</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>作り置きの蒸し鶏を使う</t>
-        </is>
-      </c>
+          <t>ゆで卵・ソテー・朝食</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>鶏肉とほうれん草のクリームシチュー</t>
+          <t>卵・大豆・乳</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>主菜+副菜</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>水夜・木昼</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/329056906922427410</t>
+          <t>木綿豆腐</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>丁</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>残りを翌昼に回す</t>
-        </is>
-      </c>
+          <t>肉豆腐</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>鮭としめじの炊き込みごはん</t>
+          <t>卵・大豆・乳</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>主食+主菜</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>木夜・金朝</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/139805641278488995</t>
+          <t>厚揚げ</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>丁</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>残りを翌朝に回す</t>
-        </is>
-      </c>
+          <t>味噌汁</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ほうれん草のおひたし</t>
+          <t>卵・大豆・乳</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>副菜</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>木夜</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/390846387756991532</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
+          <t>納豆</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>パック</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>朝食</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>肉豆腐</t>
+          <t>卵・大豆・乳</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>主菜</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>金夜</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/194111675098464660</t>
+          <t>牛乳 1L</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>本</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>リンクは牛肉。豚でも可</t>
-        </is>
-      </c>
+          <t>シチュー・朝食</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>豚肉とさつまいもの味噌汁</t>
+          <t>卵・大豆・乳</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>汁物</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>土昼</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/180204471723229588</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
+          <t>無糖ヨーグルト 400g</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>個</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>朝食・間食</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>塩サバの味噌煮</t>
+          <t>卵・大豆・乳</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>主菜</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>土夜</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/525069606923010402</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr"/>
+          <t>スライスチーズ</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>袋</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>朝食・間食</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>野菜</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>じゃがいも</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>個</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>肉じゃが・シチュー</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>補足リンク</t>
-        </is>
-      </c>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>野菜</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>にんじん</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>本</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>肉じゃが・筑前煮・シチュー</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>冷凍ブロッコリーの解凍方法</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/recipes/419552908254642504</t>
-        </is>
-      </c>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>野菜</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>玉ねぎ</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>個</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>肉じゃがほか</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>冷凍ブロッコリー活用レシピ19選</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/curations/7597</t>
-        </is>
-      </c>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>野菜</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>さつまいも</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>本</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>味噌汁</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>冷凍ブルーベリーレシピ</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>https://delishkitchen.tv/articles/31</t>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>野菜</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>白菜</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>個</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>味噌汁</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>野菜</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>ほうれん草</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>袋</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>ソテー・シチュー・おひたし</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>野菜</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>ごぼう</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>本</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>筑前煮</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>野菜</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>れんこん</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>節</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>筑前煮</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>野菜</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>里芋</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>個</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>筑前煮</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>野菜</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>こんにゃく</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>枚</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>筑前煮</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>野菜</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>長ねぎ</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>本</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>肉豆腐・蒸し鶏ごはん</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>野菜</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>しめじ</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>パック</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>炊き込みごはん・シチュー</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>野菜</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>いんげん</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>袋</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>肉じゃが</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>冷凍・乾物</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>冷凍ブロッコリー</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>450</v>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>副菜</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>冷凍・乾物</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>冷凍ブルーベリー</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>300</v>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>朝食・間食</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>冷凍・乾物</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>干ししいたけ</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>個</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>筑前煮</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>果物</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>バナナ</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>房</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>朝食・間食</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>主食</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>米</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>毎食</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>主食</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>食パン</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>袋</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>朝食・夕食</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>主食</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>焼きのり</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>袋</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>おにぎり</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>調味料</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>味噌・顆粒だし・しょうゆ・みりん・酒・砂糖・塩こしょう</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>在庫を確認</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>調味料</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>薄力粉・バター・オリーブオイル・しょうが</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>式</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>在庫を確認</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>品目数</t>
+        </is>
+      </c>
+      <c r="B39" s="6">
+        <f>COUNTA(B2:B37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>購入済</t>
+        </is>
+      </c>
+      <c r="B40" s="6">
+        <f>COUNTIF(F2:F37,"○")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>残り</t>
+        </is>
+      </c>
+      <c r="B41" s="6">
+        <f>B39-B40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>数量は2人分の概算(Claudeの推定)。在庫を差し引いて調整。F列に○を入れると集計される。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId17"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1375,11 +1948,451 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>日付</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>曜日</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>朝</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>昼</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>夜</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>間食</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>10/23</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>金</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>ご飯 / 卵と豆腐の味噌汁 / 納豆</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>きんぴらごぼう / おにぎり / 味噌汁</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>ぶり大根 / ほうれん草のごま和え / ご飯</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>ヨーグルト+冷凍ブルーベリー</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>10/24</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>土</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>トースト / ヨーグルト+冷凍ブルーベリー / バナナ</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>豚汁 / おにぎり</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>おろし煮込みハンバーグ / 里芋の煮っころがし / ご飯</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>バナナ</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>10/25</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>日</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>ご飯 / ゆで卵 / 味噌汁</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>鶏むねの照り焼き / 冷凍ブロッコリー / ご飯</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>鶏ごぼうの炊き込みごはん / 味噌汁 / きんぴらごぼう</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>チーズ・ナッツ</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>10/26</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>月</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>トースト / チーズ / 牛乳 / バナナ</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>炊き込みご飯の残り / ゆで卵 / 里芋の煮っころがし</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>ロールキャベツ / ご飯 / 冷凍ブロッコリー</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>ヨーグルト+ブルーベリー</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>10/27</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>火</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>ご飯 / 納豆 / 味噌汁</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>ロールキャベツの残り / ご飯</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>鮭のちゃんちゃん焼き / ご飯</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>バナナ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>10/28</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>水</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>ご飯 / ゆで卵 / ヨーグルト+冷凍ブルーベリー</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>基本の親子丼 / きんぴらごぼう</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>鶏むねのポン酢照り焼き / 冷凍ブロッコリー / ご飯 / 味噌汁</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>ナッツ・牛乳</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>10/29</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>木</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>トースト / 卵 / 牛乳</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>余り物・惣菜</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>千切り野菜のだし豚しゃぶ / ご飯</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>―</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>来週=10/23(金)〜10/29(木)。作り置きは10/22(木)。量は本人の食欲に合わせる。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>順</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>品名</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>目安</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>使う日</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>メモ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>ご飯を炊いて小分け冷凍</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>約5合</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>毎食</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>最初に炊飯器をセット(提案)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>きんぴらごぼう</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>約4人分</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>金昼・日夜・水昼</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>木曜に作る</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>里芋の煮っころがし</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>約4人分</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>土夜・月昼</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>下ゆでしてぬめりを取る</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>ゆで卵</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>6個</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>日朝・月昼ほか</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>―</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>保存日数が記載されていない品は早めに食べ切る。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="38" customWidth="1" min="5" max="5"/>
@@ -1426,23 +2439,23 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>鶏むね肉</t>
+          <t>ぶり 切り身</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>枚</t>
+          <t>切れ</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>蒸し鶏</t>
-        </is>
-      </c>
-      <c r="F2" s="8" t="n"/>
+          <t>ぶり大根</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1452,23 +2465,23 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>鶏もも肉</t>
+          <t>豚ひき肉</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>枚</t>
+          <t>g</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>筑前煮・クリームシチュー</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="n"/>
+          <t>おろし煮込みハンバーグ</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1478,11 +2491,11 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>牛または豚の切り落とし</t>
+          <t>合いびき肉</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>350</v>
+        <v>150</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -1491,10 +2504,10 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>肉じゃが・肉豆腐</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="n"/>
+          <t>ロールキャベツ</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1504,23 +2517,23 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>豚こま切れ</t>
+          <t>鶏むね肉</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>枚</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>豚肉とさつまいもの味噌汁</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="n"/>
+          <t>照り焼き・ポン酢照り焼き</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1530,23 +2543,23 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>タラ 切り身</t>
+          <t>鶏もも肉</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>切れ</t>
+          <t>枚</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>ムニエル</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="n"/>
+          <t>炊き込みごはん・親子丼</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1556,23 +2569,23 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>生鮭 切り身</t>
+          <t>豚こま切れ</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>切れ</t>
+          <t>g</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>炊き込みごはん</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="n"/>
+          <t>豚汁</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1582,49 +2595,49 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>塩サバ</t>
+          <t>豚ロースしゃぶしゃぶ用</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>切れ</t>
+          <t>g</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>味噌煮</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="n"/>
+          <t>だし豚しゃぶ</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>卵・大豆・乳</t>
+          <t>肉・魚</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>卵</t>
+          <t>生鮭 切り身</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>個</t>
+          <t>切れ</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>ゆで卵・ソテー・朝食</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="n"/>
+          <t>ちゃんちゃん焼き</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1634,23 +2647,23 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>木綿豆腐</t>
+          <t>卵</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>丁</t>
+          <t>個</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>肉豆腐</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="n"/>
+          <t>ゆで卵・親子丼ほか</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1660,7 +2673,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>厚揚げ</t>
+          <t>絹豆腐</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -1676,7 +2689,7 @@
           <t>味噌汁</t>
         </is>
       </c>
-      <c r="F11" s="8" t="n"/>
+      <c r="F11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1702,7 +2715,7 @@
           <t>朝食</t>
         </is>
       </c>
-      <c r="F12" s="8" t="n"/>
+      <c r="F12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1725,10 +2738,10 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>シチュー・朝食</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="n"/>
+          <t>朝食・ロールキャベツ</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1754,7 +2767,7 @@
           <t>朝食・間食</t>
         </is>
       </c>
-      <c r="F14" s="8" t="n"/>
+      <c r="F14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1780,7 +2793,7 @@
           <t>朝食・間食</t>
         </is>
       </c>
-      <c r="F15" s="8" t="n"/>
+      <c r="F15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1790,23 +2803,23 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>じゃがいも</t>
+          <t>大根</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>個</t>
+          <t>本</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>肉じゃが・シチュー</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="n"/>
+          <t>ぶり大根・豚汁・おろし煮込みほか</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1816,11 +2829,11 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>にんじん</t>
+          <t>ごぼう</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -1829,10 +2842,10 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>肉じゃが・筑前煮・シチュー</t>
-        </is>
-      </c>
-      <c r="F17" s="8" t="n"/>
+          <t>きんぴら・豚汁・炊き込み</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1842,7 +2855,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>玉ねぎ</t>
+          <t>にんじん</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
@@ -1850,15 +2863,15 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>個</t>
+          <t>本</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>肉じゃがほか</t>
-        </is>
-      </c>
-      <c r="F18" s="8" t="n"/>
+          <t>きんぴら・豚汁ほか</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1868,23 +2881,23 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>さつまいも</t>
+          <t>里芋</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>本</t>
+          <t>個</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>味噌汁</t>
-        </is>
-      </c>
-      <c r="F19" s="8" t="n"/>
+          <t>煮っころがし</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1894,11 +2907,11 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>白菜</t>
+          <t>キャベツ</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -1907,10 +2920,10 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>味噌汁</t>
-        </is>
-      </c>
-      <c r="F20" s="8" t="n"/>
+          <t>ロールキャベツ・ちゃんちゃん焼き・豚しゃぶ</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1920,7 +2933,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>ほうれん草</t>
+          <t>玉ねぎ</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
@@ -1928,15 +2941,15 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>袋</t>
+          <t>個</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>ソテー・シチュー・おひたし</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="n"/>
+          <t>ハンバーグ・ロールキャベツほか</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1946,7 +2959,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>ごぼう</t>
+          <t>ほうれん草</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
@@ -1954,15 +2967,15 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>本</t>
+          <t>袋</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>筑前煮</t>
-        </is>
-      </c>
-      <c r="F22" s="8" t="n"/>
+          <t>ごま和え</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1972,23 +2985,23 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>れんこん</t>
+          <t>長ねぎ</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>節</t>
+          <t>本</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>筑前煮</t>
-        </is>
-      </c>
-      <c r="F23" s="8" t="n"/>
+          <t>豚汁ほか</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1998,23 +3011,23 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>里芋</t>
+          <t>しょうが</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>個</t>
+          <t>かけ</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>筑前煮</t>
-        </is>
-      </c>
-      <c r="F24" s="8" t="n"/>
+          <t>ぶり大根</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2037,72 +3050,72 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>筑前煮</t>
-        </is>
-      </c>
-      <c r="F25" s="8" t="n"/>
+          <t>豚汁</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>野菜</t>
+          <t>冷凍・乾物</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>長ねぎ</t>
+          <t>冷凍ブロッコリー</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>2</v>
+        <v>450</v>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>本</t>
+          <t>g</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>肉豆腐・蒸し鶏ごはん</t>
-        </is>
-      </c>
-      <c r="F26" s="8" t="n"/>
+          <t>副菜</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>野菜</t>
+          <t>冷凍・乾物</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>しめじ</t>
+          <t>冷凍ブルーベリー</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>2</v>
+        <v>300</v>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>パック</t>
+          <t>g</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>炊き込みごはん・シチュー</t>
-        </is>
-      </c>
-      <c r="F27" s="8" t="n"/>
+          <t>朝食・間食</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>野菜</t>
+          <t>果物</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>いんげん</t>
+          <t>バナナ</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
@@ -2110,103 +3123,103 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>袋</t>
+          <t>房</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>肉じゃが</t>
-        </is>
-      </c>
-      <c r="F28" s="8" t="n"/>
+          <t>朝食・間食</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>冷凍・乾物</t>
+          <t>主食</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>冷凍ブロッコリー</t>
+          <t>米</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>450</v>
+        <v>1.5</v>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>副菜</t>
-        </is>
-      </c>
-      <c r="F29" s="8" t="n"/>
+          <t>毎食</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>冷凍・乾物</t>
+          <t>主食</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>冷凍ブルーベリー</t>
+          <t>食パン</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>300</v>
+        <v>1</v>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>袋</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>朝食・間食</t>
-        </is>
-      </c>
-      <c r="F30" s="8" t="n"/>
+          <t>朝食</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>冷凍・乾物</t>
+          <t>主食</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>干ししいたけ</t>
+          <t>焼きのり</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>個</t>
+          <t>袋</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>筑前煮</t>
-        </is>
-      </c>
-      <c r="F31" s="8" t="n"/>
+          <t>おにぎり</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>果物</t>
+          <t>調味料</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>バナナ</t>
+          <t>味噌・顆粒だし・しょうゆ・みりん・酒・砂糖・塩こしょう・米</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
@@ -2214,181 +3227,77 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>房</t>
+          <t>式</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>朝食・間食</t>
-        </is>
-      </c>
-      <c r="F32" s="8" t="n"/>
+          <t>在庫を確認</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>調味料</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>米</t>
+          <t>白すりごま・ごま油・片栗粉・パン粉・ポン酢・コンソメ</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>式</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>毎食</t>
-        </is>
-      </c>
-      <c r="F33" s="8" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>主食</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>食パン</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>袋</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>朝食・夕食</t>
-        </is>
-      </c>
-      <c r="F34" s="8" t="n"/>
+          <t>在庫を確認</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>主食</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>焼きのり</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>袋</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>おにぎり</t>
-        </is>
-      </c>
-      <c r="F35" s="8" t="n"/>
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>品目数</t>
+        </is>
+      </c>
+      <c r="B35" s="6">
+        <f>COUNTA(B2:B33)</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>調味料</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>味噌・顆粒だし・しょうゆ・みりん・酒・砂糖・塩こしょう</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>式</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>在庫を確認</t>
-        </is>
-      </c>
-      <c r="F36" s="8" t="n"/>
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>購入済</t>
+        </is>
+      </c>
+      <c r="B36" s="6">
+        <f>COUNTIF(F2:F33,"○")</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>調味料</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>薄力粉・バター・オリーブオイル・しょうが</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>式</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>在庫を確認</t>
-        </is>
-      </c>
-      <c r="F37" s="8" t="n"/>
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>残り</t>
+        </is>
+      </c>
+      <c r="B37" s="6">
+        <f>B35-B36</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>品目数</t>
-        </is>
-      </c>
-      <c r="B39" s="6">
-        <f>COUNTA(B2:B37)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t>購入済</t>
-        </is>
-      </c>
-      <c r="B40" s="6">
-        <f>COUNTIF(F2:F37,"○")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>残り</t>
-        </is>
-      </c>
-      <c r="B41" s="6">
-        <f>B39-B40</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>数量は2人分の概算(Claudeの推定)。在庫を差し引いて調整。F列に○を入れると集計される。</t>
         </is>
@@ -2399,7 +3308,977 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>週</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>料理名</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>役割</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>使う日</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>出典(デリッシュキッチン)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>メモ</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>今週</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>筑前煮</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>主菜+副菜(作り置き)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>土昼</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/202971540197736870</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>日曜に作る。干ししいたけの戻し汁を煮汁に使う</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>今週</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>蒸し鶏(生姜風味・レンジ)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>主菜(作り置き)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>金昼・日昼</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/149665586794725670</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>鶏むね肉を使用</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>今週</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>さつまいもと厚揚げの味噌汁</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>汁物</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>金朝</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/379110584001496297</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>今週</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>肉じゃが(基本)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>主菜+副菜</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>金夜・火昼</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/153240773708480781</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>残りを翌昼に回す</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>今週</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>ほうれん草と卵のソテー</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>副菜</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>金夜</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/337352711349470342</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>今週</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>タラのムニエル</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>主菜</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>土夜</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/357472571177829394</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>今週</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>白菜とさつまいもの味噌汁</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>汁物</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>日朝</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/173108175090745836</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>今週</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>カオマンガイ風 蒸し鶏ごはん</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>主食+主菜</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>日昼</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/292861887203246397</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>作り置きの蒸し鶏を使う</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>今週</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>鶏肉とほうれん草のクリームシチュー</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>主菜+副菜</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>日夜・月昼</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/329056906922427410</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>残りを翌昼に回す</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>今週</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>鮭としめじの炊き込みごはん</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>主食+主菜</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>月夜・火朝</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/139805641278488995</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>残りを翌朝に回す</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>今週</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>ほうれん草のおひたし</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>副菜</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>月夜</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/390846387756991532</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>今週</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>肉豆腐</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>主菜</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>火夜</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/194111675098464660</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>リンクは牛肉。豚でも可</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>今週</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>豚肉とさつまいもの味噌汁</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>汁物</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>水昼</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/180204471723229588</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>今週</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>塩サバの味噌煮</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>主菜</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>水夜</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/525069606923010402</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>来週</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>きんぴらごぼう(基本)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>副菜(作り置き)</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>金昼・日夜・水昼</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/143452682072359331</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>木曜に作る</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>来週</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>里芋の煮っころがし</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>副菜(作り置き)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>土夜・月昼</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/198044984757191078</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>木曜に作る。下ゆでしてぬめりを取る</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>来週</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>卵と豆腐の味噌汁</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>汁物</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>金朝</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/372431553340376263</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>来週</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>ぶり大根</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>主菜+副菜</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>金夜</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/184834780083257766</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>大根は米と下ゆで</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>来週</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>ほうれん草のごま和え(レンジ)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>副菜</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>金夜</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/134723216676487553</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>来週</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>豚汁</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>汁物</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>土昼</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/197484660219969894</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>豚バラは豚こまに替えてもよい(提案)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>来週</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>おろし煮込みハンバーグ</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>主菜</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>土夜</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/171970343445987820</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>大根おろしの水気を切る</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>来週</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>鶏むねの照り焼き(冷めても柔らか)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>主菜</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>日昼</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/118520140160565572</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>来週</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>鶏肉とごぼうの甘辛炊き込みごはん</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>主食+主菜</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>日夜・月昼</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/212230200996397460</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>3合炊き用。残りを月昼に</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>来週</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>基本のロールキャベツ</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>主菜+副菜</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>月夜・火昼</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/167621108617445868</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>煮込みすぎない</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>来週</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>鮭のちゃんちゃん焼き(フライパン)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>主菜+副菜</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>火夜</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/313873402844676537</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>来週</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>基本の親子丼</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>主食+主菜</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>水昼</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/197320405118092320</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>来週</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>鶏むねのポン酢照り焼き</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>主菜</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>水夜</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/250934092239996126</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>来週</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>千切り野菜のだし豚しゃぶ</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>主菜+副菜</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>木夜</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/433714990541701537</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>補足リンク</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>冷凍ブロッコリーの解凍方法</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/recipes/419552908254642504</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>冷凍ブロッコリー活用レシピ19選</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/curations/7597</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>冷凍ブルーベリーレシピ</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>https://delishkitchen.tv/articles/31</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId31"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2430,7 +4309,7 @@
           <t>主食+主菜+副菜をそろえると栄養がととのいやすい</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>https://www.city.bunkyo.lg.jp/documents/1540/2024321215312.pdf</t>
         </is>
@@ -2442,7 +4321,7 @@
           <t>授乳中は妊娠前より約350kcal・たんぱく質約20gの上乗せが勧められる</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>https://www.med.jrc.or.jp/Portals/0/resources/hospital/clinic/sanka/eiyo.pdf</t>
         </is>
@@ -2454,7 +4333,7 @@
           <t>鉄はビタミンCと一緒に。和食中心・脂っこい物と菓子は控えめ・水分補給</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>https://www.kenko-shokuiku.city.nagoya.jp/pdf/ninsanpu_syokuji.pdf</t>
         </is>
@@ -2466,7 +4345,7 @@
           <t>日本人の食事摂取基準(2025年版)公式</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>https://www.mhlw.go.jp/content/10904750/001542297.pdf</t>
         </is>
@@ -2478,7 +4357,7 @@
           <t>冷凍野菜の栄養(生より少ないビタミンCもある)</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>https://hugkum.sho.jp/402470</t>
         </is>

</xml_diff>